<commit_message>
NETPLY v6 : contenu retravaillé d'après TITAPLY EC (sans écraser l'existant)
Nouvelle version (netply-v6.json → Fiche technique NETPLY v6.html), l'actuelle
et le gabarit/ancre d'identité restent intacts.
- Specs CORRIGÉES d'après la fiche 2018 : acier galvanisé, média synthétique
  sans couture ni colle, 2× surface frontale, M1, 60 °C, 100 %, ΔP finale
  200 Pa (ISO) / init+50 (EN13053) — l'ancien gabarit indiquait par erreur
  plastique ABS / cadre carton.
- Descriptif reformulé, positionnement éco-conception GÉNÉRIQUE (pas de
  revendication du brevet Titanair).
- Photo TITAPLY EC réelle détourée sur blanc (croissance de région).
- Bibliothèque : NETPLY → v6.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -787,18 +787,22 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>v4</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr"/>
+          <t>v6</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Validée</t>
+          <t>Créée — G4+M5 (polynôme)</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Fiche technique NETPLY v4.html</t>
+          <t>Fiches_Netair/Fiche technique NETPLY v6.html</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -808,7 +812,7 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>Seule fiche déjà rédigée — base de référence visuelle · Données alignées sur la fiche v4</t>
+          <t>v6 retravaillée d'après TITAPLY EC (fiche 2018) : specs corrigées (acier galvanisé, sans couture ni colle), éco-conception générique. v1.0 (gabarit) conservée comme ancre d'identité.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fiche technique NETMETAL (mono-classe G3 / Coarse 50%)
Cellule filtrante métallique régénérable (équiv. Titanair TITAMETAL KMZ/A,
média aluminium ép. 48 mm). Données réelles fiche 2018 FT 2019-037 :
EN779 G3, ISO Coarse 50%, M0, T° 150 °C (acc. 200 °C/1 h), ΔP finale 250 Pa.

- Courbe ΔP = cache graphe Excel KMZA Ep48 (12/19/28/39/53 Pa à 0,79→2,38 m/s)
- Polynôme ajusté 7,34·v²+2,44·v+5,57 (fit 5 pts, R²≈1)
- Vmax 2,4 · nominal 1,5 m/s (1900 m³/h, ΔP nom ≈26 Pa), dans la plage mesurée
- Arbitrage sources : doc 2015 G1-G2 vs fiches 2018 G3 → priorité fiche 2018
- Descriptif reformulé ; photo Titanair détourée sur blanc (placeholder à remplacer)
- MAJ sources de vérité : DONNEES_PDC (ligne NETMETAL) + Bibliothèque + PROCESS
- Test d'identité NETPLY : OK (moteur inchangé)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -639,28 +639,44 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>G1 / G2</t>
+          <t>G3 (réf.) — gamme G1 → G3</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>ISO Coarse</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr"/>
+          <t>Coarse 50%</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J4" s="7" t="inlineStr"/>
+          <t>Créée — mono-classe G3 (photo placeholder à remplacer)</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETMETAL.html</t>
+        </is>
+      </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
           <t>TITAMETAL</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr"/>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>Mono-classe G3 / Coarse 50% d'après fiche 2018 TITAMETAL KMZ/A (média alu, ép. 48 mm) — FT 2019-037. Doc 2015 annonçait G1-G2 → priorité fiche 2018. Polynôme 7,34·v²+2,44·v+5,57 (fit 5 pts 0,79–2,38 m/s, R²≈1). Vmax 2,4 · nominal 1,5 m/s (1900 m³/h). Épaisseurs 25/30/48 ; variantes galva (KMZ) et inox 304 (KMXCA) sur demande. T° 150 °C (acc. 200 °C/1h), feu M0, régénérable. Photo Titanair détourée = placeholder à remplacer.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Fiche technique NETFIL (mono-classe G3 / Coarse 50%)
Cellule filtrante cousue (équiv. Titanair TITAFIL). Arbitrage 3 révisions :
descriptif 2015 G2/G3 · fiche v2_2020 G3 · v3_2023 G4/Coarse 65%.
→ G3 retenu (cohérent gamme, sous NETPLAN/NETPLY), courbe G3 v2_2020.

- Courbe ΔP = cache graphe Excel v2_2020 [2;2,8;4;6,5;11,5;21] à 0,16–1,5 m/s
- Polynôme ajusté 3,99·v²+7,24·v+0,97 (fit 6 pts, R²≈0,994)
- Vmax 1,5 (filtre basse vitesse), pmax 24, nominal 1,0 m/s (1260 m³/h, ΔP≈12 Pa)
- Descriptif reformulé ; cadre fil acier galvanisé Ø4,5mm ; M1, 60 °C (acc. 80 °C/1h)
- Photo Titanair détourée sur blanc (placeholder à remplacer) ; épaisseur 20 mm À VALIDER
- MAJ sources de vérité : DONNEES_PDC + Bibliothèque + PROCESS (avancement)
- Domaine basse vitesse hors grille débits DONNEES_PDC → coeffs consignés en statique

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -701,28 +701,44 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>G2 / G3</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>ISO Coarse</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="6" t="inlineStr"/>
+          <t>Coarse 50%</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="inlineStr"/>
+          <t>Créée — mono-classe G3 (épaisseur &amp; photo à valider)</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETFIL.html</t>
+        </is>
+      </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
           <t>TITAFIL</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Mono-classe G3 / Coarse 50% (équivalence indicative). 3 révisions Titanair : descriptif 2015 G2/G3 ; fiche v2_2020 G3 (fibre synthétique) ; v3_2023 G4/Coarse 65% (100% polyester). Choix : G3 cohérent gamme (sous NETPLAN/NETPLY), courbe v2_2020 [2;2,8;4;6,5;11,5;21] à 0,16–1,5 m/s. Polynôme 3,99·v²+7,24·v+0,97 (fit 6 pts, R²≈0,994). Vmax 1,5 (filtre basse vitesse, ventilo-convecteurs), nominal 1,0 m/s (1260 m³/h, ΔP≈12 Pa). Cadre fil acier galvanisé Ø4,5mm. T° 60 °C (acc. 80 °C/1h), feu M1. ÉPAISSEUR 20 mm = À VALIDER (cousu sur mesure). Photo Titanair placeholder (blanc-sur-blanc) à remplacer.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">

</xml_diff>

<commit_message>
NETFIL : retrait des dimensions standard + profondeur 4,5 mm
- Moteur : nouvelle option "no_dimensions" (retire titre+table+note dimensions) ;
  format français de l'épaisseur en légende (_frnum) → "4,5 mm". Identité NETPLY OK.
- NETFIL : pas de dimensions standard (filtre cousu sur mesure) → bloc retiré.
  Profondeur corrigée à 4,5 mm (= Ø du fil du cadre, au lieu de 20 mm).
- MAJ DONNEES_PDC (ép. 4,5) + Bibliothèque (note).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -721,7 +721,7 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>Créée — mono-classe G3 (épaisseur &amp; photo à valider)</t>
+          <t>Créée — mono-classe G3 (photo à remplacer)</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>Mono-classe G3 / Coarse 50% (équivalence indicative). 3 révisions Titanair : descriptif 2015 G2/G3 ; fiche v2_2020 G3 (fibre synthétique) ; v3_2023 G4/Coarse 65% (100% polyester). Choix : G3 cohérent gamme (sous NETPLAN/NETPLY), courbe v2_2020 [2;2,8;4;6,5;11,5;21] à 0,16–1,5 m/s. Polynôme 3,99·v²+7,24·v+0,97 (fit 6 pts, R²≈0,994). Vmax 1,5 (filtre basse vitesse, ventilo-convecteurs), nominal 1,0 m/s (1260 m³/h, ΔP≈12 Pa). Cadre fil acier galvanisé Ø4,5mm. T° 60 °C (acc. 80 °C/1h), feu M1. ÉPAISSEUR 20 mm = À VALIDER (cousu sur mesure). Photo Titanair placeholder (blanc-sur-blanc) à remplacer.</t>
+          <t>Mono-classe G3 / Coarse 50% (équivalence indicative). 3 révisions Titanair : descriptif 2015 G2/G3 ; fiche v2_2020 G3 (fibre synthétique) ; v3_2023 G4/Coarse 65% (100% polyester). Choix : G3 cohérent gamme (sous NETPLAN/NETPLY), courbe v2_2020 [2;2,8;4;6,5;11,5;21] à 0,16–1,5 m/s. Polynôme 3,99·v²+7,24·v+0,97 (fit 6 pts, R²≈0,994). Vmax 1,5 (filtre basse vitesse, ventilo-convecteurs), nominal 1,0 m/s (1260 m³/h, ΔP≈12 Pa). Cadre fil acier galvanisé Ø4,5mm. T° 60 °C (acc. 80 °C/1h), feu M1. Profondeur ≈ 4,5 mm (Ø fil du cadre) ; pas de dimensions standard (cousu sur mesure) → bloc dimensions retiré. Photo Titanair placeholder (blanc-sur-blanc) à remplacer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fiche technique NETFIBRE — mono-classe G4 (panneau découpé sur mesure)
- Génération via Generateur/ (gabarit NETPLY intact, test d'identité OK)
- Sources : fiche 2018 TITAFIBRE G4 (FT 2018-030, ép. 20 mm, courbe ΔP
  [12;25;41;68]) + descriptif reformulé doc 2015. Polynôme 14·v²+1,8·v+8
  (fit 4 pts, R²≈0,998), Vmax 2 · nominal 1,5 m/s (1900 m³/h, ΔP≈42 Pa).
- Contrôle : courbe G4 identique à NETPLAN (graphe Excel réutilisé) mais
  recoupée par doc 2013 (ΔP init G4 38 Pa @1,5 m/s) → retenue, signalée.
- no_dimensions (100% sur mesure) + surface_facteur 1 ; mention rouleau
  20×2 m. Gamme G2→M5 annoncée, courbes G2/G3/M5 à mesurer.
- MàJ sources de vérité : DONNEES_PDC r9, Bibliothèque r6, PROCESS.md.
- Photo Titanair détourée sur blanc (placeholder à remplacer).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -758,7 +758,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Rouleau media synthétique</t>
+          <t>Média synthétique (panneau découpé)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -771,20 +771,36 @@
           <t>ISO Coarse → ePM10</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J6" s="7" t="inlineStr"/>
+          <t>Créée — mono-classe G4 (photo Titanair détourée, à remplacer)</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETFIBRE.html</t>
+        </is>
+      </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
           <t>TITAFIBRE</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr"/>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>Mono-classe G4 / Coarse 65% (réf.) d'après fiche 2018 TITAFIBRE G4 (FT 2018-030, ép. 20 mm). Commercialisé en PANNEAU DÉCOUPÉ sur mesure (média aussi en rouleau 20×2 m), pas de tableau dimensions. Courbe ΔP [12;25;41;68] à v[0,5;1;1,5;2] = identique à NETPLAN (probable graphe Excel réutilisé) mais recoupée par doc 2013 (ΔP init G4 38 Pa @1,5 m/s) → retenue. Polynôme 14·v²+1,8·v+8 (fit 4 pts, R²≈0,998). Vmax 2, nominal 1,5 m/s (1900 m³/h, ΔP≈42 Pa). T° 80 °C (acc. 85 °C/1h), feu M1, lavable 2-3× (séries G). Gamme complète G2→M5 annoncée (specs+sous-titre) mais courbes G2/G3/M5 à mesurer (1 point doc 2013 : G2 10/G3 24/M5 125 Pa @1,5 m/s).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">

</xml_diff>

<commit_message>
NETPLY : consolidation — la v6 devient la fiche officielle (v1.0)
- "Fiche technique NETPLY.html" = ex-v6 (specs réelles TITAPLY EC), pied de
  page v1.0 ; ancienne fiche placeholder archivée dans _Archive/divers/.
- produits/netply.json = fiche produit officielle ; l'ancre du test
  d'identité est désormais produits/_gabarit_ref.json (clarifié).
- Doc (PROCESS.md, README) + Bibliothèque mises à jour.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -835,7 +835,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>v6</t>
+          <t>v1.0</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -845,12 +845,12 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Créée — G4+M5 (polynôme)</t>
+          <t>Validée — G4+M5 (polynôme)</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Fiches_Netair/Fiche technique NETPLY v6.html</t>
+          <t>Fiches_Netair/Fiche technique NETPLY.html</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>v6 retravaillée d'après TITAPLY EC (fiche 2018) : specs corrigées (acier galvanisé, sans couture ni colle), éco-conception générique. v1.0 (gabarit) conservée comme ancre d'identité.</t>
+          <t>Fiche officielle (ex-v6) d'après TITAPLY EC : specs réelles, éco-conception. Ancienne fiche placeholder archivée. Ancre test d'identité = produits/_gabarit_ref.json.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETBAG S : fiche poches souples multi-classes (moteur N-séries)
- Nouveau mode `series` opt-in dans generer.py : courbe N classes
  (M5→F9) × longueurs de poche + calculateur à sélecteur classe/longueur.
  Chemin legacy 2×2 inchangé → test d'identité NETPLY préservé (diff vide).
- 10 courbes ΔP RÉELLES extraites des courbes vectorielles des PDF
  TITABAG 2018 (recalées sur axes ; contrôle F9 p500 = 38..199 Pa),
  polynômes a·v²+b·v+c (R²≈1), surface média réelle par ligne (3,46–6,10 m²).
- Descriptif reformulé du livret_2023 ; specs fiches 2018 (T° 60°C, M1,
  écarteurs thermosoudés sans colle, cadre acier galva/PP). ADD +100 Pa (ePM).
- Anomalie M5 550 vs 650 signalée (« à valider », pointillé).
- MAJ DONNEES_PDC (l.28-37, polynômes auto LINEST), Bibliothèque, PROCESS.
- CHECKLIST_NETBAG.md pour les éléments manquants. Photo = placeholder détouré.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -949,28 +949,44 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>G4 → F9</t>
+          <t>M5 → F9 (+ G4)</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>ePM10 → ePM1</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr"/>
-      <c r="H9" s="6" t="inlineStr"/>
+          <t>ePM10 50% → ePM1 80%</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="inlineStr"/>
+          <t>Créée — multi-classes M5→F9 (courbe N-séries, photo placeholder)</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETBAG S.html</t>
+        </is>
+      </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
           <t>TITABAG S</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>Fiche MULTI-CLASSES (moteur 'series' opt-in). 10 courbes ΔP réelles extraites des courbes vectorielles des PDF TITABAG 2018 (recalées axes ; F9 p500 = contrôle 38..199 Pa). Classes M5/M6/F7/F8/F9 × profondeurs 380/500/550/650 ; surface média réelle par ligne (3,46–6,10 m²). Toutes ePM → ADD +100 Pa. Anomalie M5 550 vs 650 (550 marquée à valider). G4 annoncé (gamme) mais non mesuré. T° 60°C, feu M1, écarteurs thermosoudés sans colle, cadre acier galva/PP ép.25. Données détail : DONNEES_PDC l.28-37. Manques : CHECKLIST_NETBAG.md. Photo Titabag détourée = placeholder.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">

</xml_diff>

<commit_message>
NETPAK S CILIA : F7 = TITAPAK S GR PRISME A (GREENTEX, ePM1 50%)
Correction demandée : le F7 prend la fiche GR PRISME A (GREENTEX, média
basse résistance) en ep48 + ep98, au lieu de la HPE (ePM1 55%).
- ep48 : 12·20·30·40·51·63·76 Pa → 2,858·v²+15,584·v−2,224 (R²=0,9999)
- ep98 : 10·19·29·40·52·67·86 Pa → 5,883·v²+7,916·v+0,756 (R²=0,999)
F7 passe à ePM1 50% ; ΔP plus faible que HPE (média green), sous M5/M6.
M5/M6/F8/F9 inchangés (HPE PRISME A). Léger croisement ep48/ep98 F7 à
haute vitesse (présent dans la fiche source).

Ajustements densité page 2 pour tenir l'A4 (paddings tableau ΔP).
Registres (DONNEES_PDC l.42-43, Bibliothèque) + PROCESS.md mis à jour.
Test d'identité NETPLY : diff vide.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1066,7 +1066,7 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>ePM10 50% → ePM1 80%</t>
+          <t>ePM10 50% → ePM1 80% (F7 = ePM1 50% GREENTEX)</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>Cadre acier galvanisé (-A) / plastique (-P). Sources PRISME A HPE 2018 (ep48+ep98). Surface m²/m². Pièges : F8=F9 en PRISME P (écarté → PRISME A) ; F9 ep48 = F8+10 Pa (offset suspect) ; F8 ep98 7e pt extrapolé. PHOTO PLACEHOLDER à remplacer.</t>
+          <t>Cadre acier galvanisé (-A) / plastique (-P). Sources PRISME A HPE 2018 (M5/M6/F8/F9) + GR PRISME A GREENTEX pour F7 (ePM1 50%, ep48+ep98). Surface m²/m². Pièges : F8=F9 en PRISME P (écarté → PRISME A) ; F9 ep48 = F8+10 Pa (offset suspect) ; F8 ep98 7e pt extrapolé. PHOTO PLACEHOLDER à remplacer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETMETAL G2/G3 + confirmations specs (NETFIL G3, NETFIBRE 60°C) ; trace débordement A4 p2
- NETMETAL : classe affichée G2 / G3 (déc. PA), courbe réf. G3 mesurée inchangée
- NETFIL G3 (v2_2020) et NETFIBRE 60 °C : choix confirmés par PA, marqués résolus
- CHECKLIST : item 🟠 débordement page 2 (~1222 px) sur les fiches 2-classes/mono
- Identité NETPLY : diff vide

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -639,7 +639,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>G3 (réf.) — gamme G1 → G3</t>
+          <t>G2 / G3</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>Mono-classe G3 / Coarse 50% d'après fiche 2018 TITAMETAL KMZ/A (média alu, ép. 48 mm) — FT 2019-037. Doc 2015 annonçait G1-G2 → priorité fiche 2018. Polynôme 7,34·v²+2,44·v+5,57 (fit 5 pts 0,79–2,38 m/s, R²≈1). Vmax 2,4 · nominal 1,5 m/s (1900 m³/h). Toutes dimensions sur mesure (pas de dimensions standard) ; épaisseurs standard 10/15/20/25/30/48 ; variantes galva (KMZ) et inox 304 (KMXCA) sur demande. T° 150 °C (acc. 200 °C/1h), feu M0, régénérable. Photo Titanair détourée = placeholder à remplacer.</t>
+          <t>Mono-classe G3 / Coarse 50% d'après fiche 2018 TITAMETAL KMZ/A (média alu, ép. 48 mm) — FT 2019-037. Doc 2015 annonçait G1-G2 → priorité fiche 2018. Polynôme 7,34·v²+2,44·v+5,57 (fit 5 pts 0,79–2,38 m/s, R²≈1). Vmax 2,4 · nominal 1,5 m/s (1900 m³/h). Toutes dimensions sur mesure (pas de dimensions standard) ; épaisseurs standard 10/15/20/25/30/48 ; variantes galva (KMZ) et inox 304 (KMXCA) sur demande. T° 150 °C (acc. 200 °C/1h), feu M0, régénérable. Photo Titanair détourée = placeholder à remplacer. Classe affichée G2 / G3 (déc. PA 22/06/2026 ; courbe réf. G3 mesurée).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETPAK S AZUR : fiche compact polydièdre (TITAPAK SV-GD)
- Fiche multi-classes F7/F8/F9 (ePM1, moteur série), profondeur 292, largeurs 592/490/287.
- Données ΔP RÉELLES : caches Excel SV-GD 2018 (F7/F9) + FORMULE_PDC. R²≈1.
  ⚠ F8 = F9×0,95 (dérivé Titanair) — affiché normalement (décision dirigeant), noté à mesurer.
  M6 ePM2,5 annoncée sans courbe → specs/badges « sur demande ». Surface média n.c.
- Moteur série : note_dimensions désormais gérée + surface « n.c. » si non fournie
  (NETPLY identité OK, NETBAG inchangé).
- MAJ DONNEES_PDC (l.48-51), Bibliothèque (l.12), CHECKLIST (section AZUR).
- Photo SV-GD réelle (© A. Périer) = placeholder. Vérifié navigateur : 3 courbes, calc
  (formule GT (finale/2)×0,85), 0 erreur JS.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1123,22 +1123,34 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>M5 → F9</t>
+          <t>F7 → F9 (M6 sur demande)</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>ePM10 → ePM1</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="6" t="inlineStr"/>
+          <t>ePM1 55% → 80%</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J12" s="7" t="inlineStr"/>
+          <t>Créée — F7/F8/F9 (moteur série, photo réelle placeholder)</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETPAK S AZUR.html</t>
+        </is>
+      </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
           <t>TITAPAK SV GD</t>
@@ -1146,7 +1158,7 @@
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>Nom produit ⚠ à valider</t>
+          <t>Compact polydièdre rigide (équiv. TITAPAK SV-GD). 3 classes ePM1 F7/F8/F9, profondeur 292, largeurs 592/490/287. Données réelles caches Excel SV-GD 2018 (F7/F9) + FORMULE_PDC. ⚠ F8 = F9×0,95 (dérivé, affiché normalement sur décision PA, à mesurer). M6 ePM2,5 50% annoncée (livret) sans courbe → specs/badges seulement. Surface média n.c. Parois polystyrène, média PP, séparateurs hot melt, M1, 60°C, EN13053 init+100. DONNEES_PDC l.48-51. Photo SV-GD réelle = placeholder. Détail : CHECKLIST.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETPAK S LUMEN : fiche compact polydièdre rechargeable (TITAPAK S QUARTZ)
- Fiche multi-classes F7/F8/F9 (ePM1, moteur série), profondeur 292, angle RSE/rechargeable (déchets ÷4).
- Données ΔP RÉELLES : courbes vectorielles PDF QUARTZ 2018 (FT 2019-041), cohérentes F7<F8<F9 (pas de piège). R²≈1.
- Specs fiches 2018 : polyester/PP, sans colle ni séparateur (HPE), M1, 60°C, HR 100%, EN13053 init+100.
- Calculateur formule GT (finale/2)×0,85. Vérifié navigateur : 3 courbes, 0 erreur JS.
- MAJ DONNEES_PDC (l.52-54), Bibliothèque (l.13), CHECKLIST (section LUMEN).
- ⚠ Variantes fournisseurs 2024-25 divergentes notées ; photo QUARTZ (Titanair visible) = placeholder.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1185,22 +1185,34 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>M5 → F9</t>
+          <t>F7 → F9</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>ePM10 → ePM1</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr"/>
-      <c r="H13" s="6" t="inlineStr"/>
+          <t>ePM1 55% → 80%</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J13" s="7" t="inlineStr"/>
+          <t>Créée — F7/F8/F9 rechargeable (moteur série, photo placeholder)</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETPAK S LUMEN.html</t>
+        </is>
+      </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
           <t>TITAPAK S QUARTZ</t>
@@ -1208,7 +1220,7 @@
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>Argument RSE — cassettes rechargeables. Nom ⚠ à valider</t>
+          <t>Compact polydièdre RECHARGEABLE (équiv. TITAPAK S QUARTZ) — argument RSE (déchets ÷4, cassettes remplacées). 3 classes ePM1 F7/F8/F9, profondeur 292. Données réelles courbes vectorielles PDF 2018 (FT 2019-041), cohérentes F7&lt;F8&lt;F9 (pas de piège). Polyester/PP, sans colle ni séparateur (HPE), M1, 60°C, HR 100%, EN13053 init+100. ⚠ Variantes MFILTER/FILTECH 2024-25 divergent → priorité 2018. % ePM1 : livret 60/90 vs fiche 55/80 (retenu). Surface média n.c. DONNEES_PDC l.52-54. Photo QUARTZ (Titanair visible) = placeholder.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETPAK S BORA : panneau compact à brides GREENTEX (TITAPAK S DSK)
- Fiche mono-classe F7 GREENTEX (ePM1 50%) — décision PA (média recyclé, angle éco).
- Données ΔP réelles lues sur l'image GR DSK F7.png (recoupées FORMULE_PDC) :
  fit 7,16·v²+11,42·v−1,13 (R²=0,9998), mesuré ≤3100 m³/h → Vmax 2,46, nominal 3000.
- Specs fiche HPE DSK 2020 : panneau 100 mm, polystyrène/PP, M1, 60°C, HR 100%,
  EN13053 init+100, technologie D.S.K. Calculateur formule GT. 0 erreur JS.
- MAJ DONNEES_PDC (l.55), Bibliothèque (l.10), CHECKLIST (section BORA).
- Variante HPE 55% non tracée (courbe non exploitable) notée. Photo DSK = placeholder.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1006,35 +1006,47 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Compact à brides</t>
+          <t>Panneau compact à brides (DSK)</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>M5 → F9</t>
+          <t>F7</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>ePM10 55% / ePM1 55%</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="6" t="inlineStr"/>
+          <t>ePM1 50% (GREENTEX)</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J10" s="7" t="inlineStr"/>
+          <t>Créée — mono-classe F7 GREENTEX (photo placeholder)</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETPAK S BORA.html</t>
+        </is>
+      </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>TITAPAK S D.S.K</t>
+          <t>TITAPAK S DSK (GR)</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>Nom produit ⚠ à valider</t>
+          <t>Panneau compact à brides 100 mm (équiv. TITAPAK S DSK). Décision PA : version GREENTEX (média recyclé, ePM1 50%) car courbe dispo et cohérente — argument éco. Courbe lue sur image GR DSK F7.png, recoupée FORMULE_PDC (polynôme GREENTEX). Fit 7,16·v²+11,42·v−1,13 (R²=0,9998), mesuré ≤3100 m³/h → Vmax 2,46, nominal 3000. Specs fiche HPE DSK 2020 : polystyrène/PP, M1, 60°C, HR 100%, technologie D.S.K (pleine surface sans préfiltre). Variante HPE ePM1 55% existe (courbe non exploitable). Surface média n.c. DONNEES_PDC l.55. Photo DSK réelle = placeholder.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETPAK S DUO : fiche combiné F7 GREENTEX + charbon actif (mono-classe, A4 OK)
Source TITAPAK S PRISME DUO F7 GR-CA ep48 (fiche 2018). Courbe ΔP réelle
combinée (36→247 Pa), polynôme 15,013·v²+28,882·v+3,537 (R²=0,9998), ΔP
nom 190 Pa. Feu NA (charbon). Bouton calculateur double efficacité, page 2
A4 OK (compact_p2), identité NETPLY verte. Registres + CHECKLIST à jour.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1591,12 +1591,12 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Combinés</t>
+          <t>Filtres combinés (NETPAK)</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Compact particulaire + charbon actif</t>
+          <t>Compact mini-plis + charbon actif</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -1606,25 +1606,37 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>ePM1 55% + Moléculaire</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr"/>
-      <c r="H21" s="6" t="inlineStr"/>
+          <t>ePM1 50% + CA</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J21" s="7" t="inlineStr"/>
+          <t>Créée — mono-classe F7 GREENTEX + charbon actif (ep48)</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETPAK S DUO.html</t>
+        </is>
+      </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>PRISME DUO</t>
+          <t>TITAPAK S PRISME DUO</t>
         </is>
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>Double filtration. Nom ⚠ à valider</t>
+          <t>F7 GREENTEX + charbon actif. ΔP combinée 36→247 Pa (nom 190). Feu NA (charbon non classé). Surface média dév. ≈12,55 m². ΔP finale +100 Pa (= règle Titanair PDC init+100). Photo placeholder PRISME A à remplacer. Capacité CA (grammage) non communiquée → R&amp;D.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETCEL V NIVAL : filtre absolu HEPA polydièdre (TITACEL V) + mode HEPA moteur
- Moteur série : option `hepa` → ΔP finale = 2 × initiale (au lieu de la règle ePM),
  note « 2 × ΔP initiale — EN 1822 ». Défaut hepa=false → fiches série existantes inchangées
  (NETBAG/AZUR/LUMEN régénérées, identité NETPLY OK).
- NIVAL : courbe H13 réelle (cache Excel TITACEL V), fit 9,44·v²+75,31·v−1,20 (R²≈1),
  surface 40 m², 610×610×292, EN 1822. E10/H14 annoncés sans courbe (H14 = copie H13 = piège) → à mesurer.
- ΔP finale HEPA = 2× initiale : recherche normes (EN 1822/ISO 29463 ne fixent rien ;
  pratique Camfil/Titanair = 2× ; CIBSE ~510 Pa). Pas d'étiquette énergie Eurovent (HEPA exclu).
- MAJ DONNEES_PDC (l.56), Bibliothèque (l.15), CHECKLIST. 0 erreur JS. Photo TITACEL V = placeholder.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1309,28 +1309,44 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>E10 → H14</t>
+          <t>E10 → H14 (EN 1822)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>ISO 35 H</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr"/>
-      <c r="H15" s="6" t="inlineStr"/>
+          <t>HEPA / T.H.E</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J15" s="7" t="inlineStr"/>
+          <t>Créée — H13 (mode HEPA, E10/H14 courbes à ajouter)</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETCEL V NIVAL.html</t>
+        </is>
+      </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
           <t>TITACEL V</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>Filtre absolu HEPA polydièdre (équiv. TITACEL V). 610×610×292, surface 40 m², média fibre de verre, M1, 60°C. Mode HEPA (ΔP finale=2×init, EN 1822 ; pas d'étiquette Eurovent). Courbe H13 réelle (cache Excel, fit 9,44·v²+75,31·v−1,20 R²≈1, ΔP@3400≈270). E10 (Excel sans cache) et H14 (courbe = copie exacte du H13, piège) annoncés mais SANS courbe → à mesurer. ⚠ 610×610 sur moteur 592×592 (axe vitesse cosmétique). DONNEES_PDC l.56. Photo TITACEL V réelle = placeholder.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1345,32 +1361,44 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>HEPA / T.H.E</t>
+          <t>HEPA / T.H.E (NETPAK)</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Filtre laminaire</t>
+          <t>HEPA terminal à flux laminaire</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>H14</t>
+          <t>H14 (EN 1822)</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>ISO 15 U</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr"/>
-      <c r="H16" s="6" t="inlineStr"/>
+          <t>≥ 99,995 % MPPS</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J16" s="7" t="inlineStr"/>
+          <t>Créée — mono-classe H14, paradigme HEPA (aref 610², ΔP finale 2×)</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETPAK V LAM.html</t>
+        </is>
+      </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
           <t>TITAPAK V LAM</t>
@@ -1378,7 +1406,7 @@
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>Pas de nom signature (volontaire). ⚠ à valider</t>
+          <t>HEPA laminaire H14. Dim. eff. 610×610×68, surface 5,83 m², média fibre de verre, cadre alu, T° 80°C, feu M1. ΔP nom ≈125 Pa @600 m³/h, finale 2× (colmatage ≈400 Pa). 1re fiche moteur en mode HEPA (aref/dim_ref/dp_final_mode x2). Photo placeholder.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETCEL V AZUR : filtre absolu HEPA multidièdre (TITAPAK V-GD)
- Fiche série mode HEPA, classes E10 + H13 (2 courbes réelles, caches Excel).
  E10 7,16·v²+56,14·v+1,33 (mesuré ≤3500) ; H13 31,80·v²+119,76·v−14,70 (24 m², ≤2400, extrapolé au-delà).
- ΔP finale = 2× initiale (EN 1822). 592×592×292, fibre de verre, M1, 60°C. 0 erreur JS.
- MAJ DONNEES_PDC (l.57-58), Bibliothèque (l.14), CHECKLIST → famille NETCEL complète (NIVAL + AZUR).
- Noté : H13 extrapolé >2400, curseur débit init 3400 (calc OK 2400), photo = idem NETPAK AZUR (à distinguer).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1259,30 +1259,42 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>E10 / H13</t>
+          <t>E10 · H13 (EN 1822)</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>ISO 50 U / ISO 35 H</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr"/>
-      <c r="H14" s="6" t="inlineStr"/>
+          <t>HEPA / T.H.E</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>22/06/2026</t>
+        </is>
+      </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J14" s="7" t="inlineStr"/>
+          <t>Créée — E10+H13 (mode HEPA)</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETCEL V AZUR.html</t>
+        </is>
+      </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>TITAPAK V GD</t>
+          <t>TITAPAK V-GD</t>
         </is>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
-          <t>Nom produit ⚠ à valider</t>
+          <t>Filtre absolu HEPA multidièdre (équiv. TITAPAK V-GD). 592×592×292, média fibre de verre, polyester, M1, 60°C. Mode HEPA (ΔP finale=2×init). Courbes réelles caches Excel : E10 7,16·v²+56,14·v+1,33 (mesuré ≤3500) ; H13 31,80·v²+119,76·v−14,70 (24 m², mesuré ≤2400, extrapolé au-delà). DONNEES_PDC l.57-58. ⚠ Photo = même polydièdre SV-GD que NETPAK S AZUR (placeholder à distinguer). Curseur débit s'init à 3400 (calc OK à 2400).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETCARB CILIA : 1re fiche charbon actif (filtration moléculaire)
Filtre compact à charbon actif (équiv. PRISME CARB), traité comme un
filtre de GAZ : cadre normatif ISO 10121 (et non ISO 16890 particules),
classe LD/MD/HD à déterminer par essai (non inventée), capacité 15% masse.
Données ΔP réelles (caches Excel 48/98 mm), polynômes 7 pts (DONNEES_PDC).

Deux options moteur additives (réutilisables famille NETCARB), sans toucher
au gabarit ni casser le test d'identité NETPLY :
- deux_epaisseurs : 1 famille × 2 épaisseurs (toggle classe masqué)
- dp_final_mode:const : filtre non colmatant (ΔP finale ≈ moyenne ≈ initiale)
- ref_simple + ΔP par ligne + en-tête « Filtration » pour le tableau dimensions

Registres à jour (Bibliothèque, DONNEES_PDC l.59-60, CHECKLIST).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1450,17 +1450,29 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Moléculaire</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr"/>
-      <c r="H17" s="6" t="inlineStr"/>
+          <t>Moléculaire (ISO 10121)</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>23/06/2026</t>
+        </is>
+      </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J17" s="7" t="inlineStr"/>
+          <t>Créée — filtre moléculaire charbon actif, 2 épaisseurs 48/98 mm</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETCARB CILIA.html</t>
+        </is>
+      </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
           <t>PRISME CARB</t>
@@ -1468,7 +1480,7 @@
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>Nom produit ⚠ à valider</t>
+          <t>Charbon actif pur (gaz) : pas de classe ePM. ISO 10121 (LD/MD/HD à déterminer). ΔP réelles caches Excel 48/98 (cohérentes 48&gt;98), poly 7 pts. ΔP non colmatante (remplacement à saturation, capacité 15% masse). T° 40°C, HR 50%, feu NA. Nouveaux drapeaux moteur deux_epaisseurs + dp_final_mode:const. Photo CARB.png (grains) placeholder.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETCARB AZUR : 2e fiche charbon actif (dièdre, mono-classe)
Poches rigides à charbon actif (équiv. SV-GD CARB), filtration moléculaire
ISO 10121, mono-classe (292 mm). Courbe 2020 « QL-CARB » retenue car
cohérente avec la fiche 2018 ; piège écarté : fichiers F7/F8 2023 = copies
du base 2023 (hors axe). Parois polyester, T° 40 °C (efficacité), HR 70 %,
capacité non communiquée → R&D.

Moteur : en-tête tableau « Filtration » rattaché à ref_simple (vaut aussi
pour les fiches charbon mono). Identité NETPLY revérifiée.

Registres à jour (Bibliothèque, DONNEES_PDC l.61, CHECKLIST, PROCESS).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1512,25 +1512,37 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Moléculaire</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr"/>
-      <c r="H18" s="6" t="inlineStr"/>
+          <t>Moléculaire (ISO 10121)</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>23/06/2026</t>
+        </is>
+      </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J18" s="7" t="inlineStr"/>
+          <t>Créée — charbon actif poches rigides/dièdre, mono-classe 292 mm</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETCARB AZUR.html</t>
+        </is>
+      </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>SV GD CARB</t>
+          <t>SV-GD CARB</t>
         </is>
       </c>
       <c r="L18" s="7" t="inlineStr">
         <is>
-          <t>Nom produit ⚠ à valider</t>
+          <t>Charbon pur (gaz), pas de classe ePM. Courbe 2020 QL-CARB (8,073·v²+13,383·v+2,929 ; ΔP@3400≈98). Piège 2023 F7=F8=base écarté. Parois POLYESTER, feu NA, T° 40°C (efficacité), HR 70%. Combinable F7/F9 option. Capacité adsorption n.c.→R&amp;D. Photo CARB_BLEND placeholder.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETCARB NIVAL : 3e fiche charbon actif (polydièdre)
Polydièdre à charbon actif (équiv. V-CARB), filtration moléculaire ISO 10121,
mono-classe 292 mm, nominal 3000. V-CARB n'ayant aucune courbe ΔP mesurée
propre, réutilise (décision PA) la courbe du pack charbon 292 mm partagée avec
AZUR (SV-GD/QL-CARB), marquée « à mesurer R&D ». Parois polyester à confirmer.

Registres à jour (Bibliothèque, DONNEES_PDC l.62, CHECKLIST, PROCESS).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1574,25 +1574,37 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Moléculaire</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr"/>
-      <c r="H19" s="6" t="inlineStr"/>
+          <t>Moléculaire (ISO 10121)</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>23/06/2026</t>
+        </is>
+      </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J19" s="7" t="inlineStr"/>
+          <t>Créée — charbon actif polydièdre, mono-classe 292 mm (courbe partagée AZUR)</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETCARB NIVAL.html</t>
+        </is>
+      </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>TITACEL CARB</t>
+          <t>V-CARB (TITACEL CARB)</t>
         </is>
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>Nom produit ⚠ à valider</t>
+          <t>Polydièdre charbon (gaz). ⚠ Aucune courbe ΔP V-CARB mesurée → courbe pack charbon 292 mm de SV-GD/QL partagée (à mesurer R&amp;D). Nominal 3000, ΔP@3000≈80. Combinable F7. T° 40°C, HR 70%, feu NA. Parois polyester à confirmer. Photo Q-carb (code visible→remplacer). Classe LD/MD/HD &amp; capacité→R&amp;D.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
NETCARB BAG : 4e fiche charbon (poches souples F9 + charbon imprégné)
Combiné particules + charbon (≠ charbon en grains) : classe ISO 16890 F9
(ePM1 80%) primaire + charbon imprégné pour odeurs/COV (capacité 15%).
Filtre colmatant → règle ΔP ePM +100 (pas la ΔP constante des grains).
Source TITABAG F9 CARB 2021, ΔP@3400 ≈ 229 Pa, profondeur 520 mm.

Famille NETCARB complète (4/4). Registres à jour (Bibliothèque, DONNEES_PDC
l.63, CHECKLIST, PROCESS — récap des 3 options moteur charbon).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1631,28 +1631,44 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>F9</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Moléculaire</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr"/>
-      <c r="H20" s="6" t="inlineStr"/>
+          <t>ePM1 80% + CA (ISO 10121)</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>v1.0</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>23/06/2026</t>
+        </is>
+      </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>À créer</t>
-        </is>
-      </c>
-      <c r="J20" s="7" t="inlineStr"/>
+          <t>Créée — poches souples F9 à charbon imprégné (combiné), mono-classe 520</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>Fiches_Netair/Fiche technique NETCARB BAG.html</t>
+        </is>
+      </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L20" s="7" t="inlineStr"/>
+          <t>TITABAG F9 CARB</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>COMBINÉ particules+charbon (≠ charbon grains) : classe ISO 16890 F9 ePM1 80% PRIMAIRE + charbon imprégné (odeurs/COV, capacité 15%). COLMATANT → règle ePM +100 (pas const). 9,172·v²+64,135·v−10,429 ; ΔP@3400≈229. Cadre acier, 520mm, T° 40°C, feu NA. HR n.c. Photo forme poches NETBAG placeholder (média imprégné à reshooter).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">

</xml_diff>

<commit_message>
NETBAG S : intégration de la classe G4 (préfiltration) en specs/gamme
G4 (Coarse 65%, EN 779) promu au rang de classe à part entière dans le
sous-titre, la description, les badges et les specs (EN 779 G4→F9, ISO
Coarse 65%, profondeur 380 mm, ΔP finale ADD +50 Coarse). Décision PA :
specs/gamme seulement, sans courbe tracée — aucune donnée ΔP G4 mesurée
n'existe (TITABAG/FORMULE_PDC) → courbe « sur demande / à mesurer R&D ».
Graphe et calculateur inchangés (M5→F9).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -954,7 +954,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>ePM10 50% → ePM1 80%</t>
+          <t>G4 · M5 · M6 · F7 · F8 · F9</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>Fiche MULTI-CLASSES (moteur 'series' opt-in). 10 courbes ΔP réelles extraites des courbes vectorielles des PDF TITABAG 2018 (recalées axes ; F9 p500 = contrôle 38..199 Pa). Classes M5/M6/F7/F8/F9 × profondeurs 380/500/550/650 ; surface média réelle par ligne (3,46–6,10 m²). Toutes ePM → ADD +100 Pa. Anomalie M5 550 vs 650 (550 marquée à valider). G4 annoncé (gamme) mais non mesuré. T° 60°C, feu M1, écarteurs thermosoudés sans colle, cadre acier galva/PP ép.25. Données détail : DONNEES_PDC l.28-37. Manques : CHECKLIST.md. Photo Titabag détourée = placeholder.</t>
+          <t>Fiche MULTI-CLASSES (moteur 'series' opt-in). 10 courbes ΔP réelles extraites des courbes vectorielles des PDF TITABAG 2018 (recalées axes ; F9 p500 = contrôle 38..199 Pa). Classes M5/M6/F7/F8/F9 × profondeurs 380/500/550/650 ; surface média réelle par ligne (3,46–6,10 m²). Toutes ePM → ADD +100 Pa. Anomalie M5 550 vs 650 (550 marquée à valider). G4 annoncé (gamme) mais non mesuré. T° 60°C, feu M1, écarteurs thermosoudés sans colle, cadre acier galva/PP ép.25. Données détail : DONNEES_PDC l.28-37. Manques : CHECKLIST.md. Photo Titabag détourée = placeholder. [MAJ 23/06: G4 (Coarse 65%, poche 380, ADD+50) intégré en specs/gamme/badges, SANS courbe — courbe G4 à mesurer (aucune donnée TITABAG/FORMULE_PDC).]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Renommage NETCEL V LAM : registres Excel (Bibliothèque + DONNEES_PDC)
Nom de gamme mis à jour dans les 2 classeurs suivis du dépôt (méthode
chirurgicale XML, contenu/formules préservés). Bibliothèque : nom + lien
fiche renommé. Cohérent avec le renommage global NETPAK V LAM → NETCEL V LAM.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1368,7 +1368,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>NETPAK V LAM</t>
+          <t>NETCEL V LAM</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>Fiches_Netair/Fiche technique NETPAK V LAM.html</t>
+          <t>Fiches_Netair/Fiche technique NETCEL V LAM.html</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Registre et PROCESS mis à jour après la passe NETMETAL v1.1
Le PROCESS impose de tenir les sources de vérité à jour à chaque fiche,
et les deux décrivaient encore l'ancien NETMETAL.

Bibliotheque : v1.0 → v1.1, date, statut « Validée PA », et la classe ISO
passe de « Coarse 50% » à « Coarse 40% / 50% » — le Coarse 40% manquait
en face du G2 pourtant annoncé.

PROCESS, état d'avancement : le repositionnement en pare-gouttelettes,
les deux dérogations à ne pas « réparer » (ΔP finale retirée de la p1,
T° laissée à 150 °C alors que l'inox tient 200 °C), les données non
sourcées confirmées par PA, et le renvoi vers _arbitrages_pad.
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -644,22 +644,22 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Coarse 50%</t>
+          <t>Coarse 40% / 50%</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>v1.0</t>
+          <t>v1.1</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>22/06/2026</t>
+          <t>17/07/2026</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>Créée — mono-classe G3 (photo placeholder à remplacer)</t>
+          <t>Validée PA — contenu retravaillé 17/07</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>Mono-classe G3 / Coarse 50% d'après fiche 2018 TITAMETAL KMZ/A (média alu, ép. 48 mm) — FT 2019-037. Doc 2015 annonçait G1-G2 → priorité fiche 2018. Polynôme 7,34·v²+2,44·v+5,57 (fit 5 pts 0,79–2,38 m/s, R²≈1). Vmax 2,4 · nominal 1,5 m/s (1900 m³/h). Toutes dimensions sur mesure (pas de dimensions standard) ; épaisseurs standard 10/15/20/25/30/48 ; variantes galva (KMZ) et inox 304 (KMXCA) sur demande. T° 150 °C (acc. 200 °C/1h), feu M0, régénérable. Photo Titanair détourée = placeholder à remplacer. Classe affichée G2 / G3 (déc. PA 22/06/2026 ; courbe réf. G3 mesurée).</t>
+          <t>Contenu validé par PA le 17/07/2026 — REPOSITIONNEMENT PRODUIT : présenté comme PARE-GOUTTELETTES (aval batteries froides) puis PARE-ÉTINCELLES (aval batteries électriques), la filtration des particules grossières devenant un usage second. Ce renversement CONTREDIT la doc Titanair 2015 (filtration en usage premier, anti-graisse/séparateur de gouttes en second) : décision PA en tant que fabricant, pas une erreur de lecture. Pare-étincelles et anti-graisse retiré : non sourcés / omis volontairement. Sous-titre « Filtre métallique » (remplace « Cellule filtrante métallique — Préfiltre régénérable ») : seule fiche de la gamme dont le sous-titre n'annonce pas le rôle. ALIGNEMENTS : ISO 16890 avant EN 779 ; ajout du Coarse 40% correspondant au G2 annoncé (il manquait ; sourcé fiches KMX/CA et WZA) ; badge ISO aligné sur le tableau (disait « Coarse 50% » seul) ; « Structure : 2 grilles métalliques » identique à NETPLY/NETPLAN (perte VOLONTAIRE de « fil zingué », pourtant sourcé doc 2015) ; cadre « inox 304 » (disait « inox » seul). DÉROGATIONS ASSUMÉES, ne pas « réparer » : (1) ligne « ΔP finale recommandée » RETIRÉE de la page 1 — seule des 18 fiches, alors que PROCESS.md la dit impérative ; le calculateur p2 applique pourtant toujours +50 Pa (il lit classes.*.add, pas la ligne specs). (2) T° 150 °C maintenue (valeur alu/galva) alors que l'inox 304 tient 200 °C continu / 300 °C acc. (KMX/CA) → variante inox volontairement sous-vendue. Épaisseurs 10/15/20 mm et HR 100 % : confirmées PA en tant que fabricant, NON SOURCÉES. Feu M0 sourcé (les 4 fiches 2018) mais classement français de 1983, remplacé par les Euroclasses EN 13501-1 (A1) + PV d'essai à sécuriser → CHECKLIST. Courbe ΔP agrandie de 21 % (nouveau drapeau courbe_large : 279 → 339 px, la plus grande de la gamme, devant NETPLY à 305). Bouton « Retour au produit » ajouté (charte, 18 fiches). TENSION OUVERTE : le calculateur p2 modélise un colmatage de filtre à particules alors que la p1 présente un pare-gouttelettes. Photo = placeholder Titanair. Détail complet : _arbitrages_pad dans netmetal.json + CHECKLIST.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Séparateur hot melt ajouté sur NETCEL V NIVAL et NETCEL V AZUR (v1.2)
Les trois fiches absolues divergeaient : LAM affichait la ligne « Séparateur »,
AZUR et NIVAL non, alors que la donnée est vraie et sourcée pour les trois. PA
tranche pour l'ajouter aux deux. Vérification faite avant écriture : les quatre
fiches source de NIVAL portent « hot melt », et les deux fiches H13 d'AZUR aussi
— sa fiche E10 n'a simplement pas le champ, ce qui ne contredit rien.

AZUR était figée en v1.1 : accord de PA obtenu, version bumpée en v1.2 et
registre aligné, 18 fiches sur 18. Contrairement au précédent du 4 août, où le
retrait de trois mots n'avait pas justifié de bump, il s'agit ici d'une ligne de
specs entière.

Les deux pages des deux fiches tiennent toujours dans l'A4, les 16 autres fiches
sont régénérées à l'octet près.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
+++ b/fiches-techniques/Bibliotheque_Fiches_Techniques_Netair.xlsx
@@ -1269,17 +1269,17 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>v1.1</t>
+          <t>v1.2</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>02/08/2026</t>
+          <t>15/08/2026</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>Validée PA — contenu retravaillé 02/08 (courbe H13 corrigée — axe débit +20 %, DONNEES_PDC réaligné ; plage E10 → H14, H14 sur devis ; nominaux 3000/2500/1500 ; boutique formats standard, classes EPA/HEPA seules) · 04/08 : « (papier HEPA) » retiré du média (déc. PA) — SANS bump de version, écart assumé</t>
+          <t>Contenu retravaillé v1.1 (02/08) — v1.2 (15/08) : ligne « Séparateur : Hot melt » ajoutée (accord PA)</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">

</xml_diff>